<commit_message>
ci(dev): publish dev build from 61babbc9c07e2cd37c38ea2d6ccf276545c8a59e 61babbc9c07e2cd37c38ea2d6ccf276545c8a59e
</commit_message>
<xml_diff>
--- a/dev/StructureDefinition-ph-core-location.xlsx
+++ b/dev/StructureDefinition-ph-core-location.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-18T03:12:48+00:00</t>
+    <t>2026-03-18T09:54:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -636,7 +636,7 @@
     <t>Location.address</t>
   </si>
   <si>
-    <t xml:space="preserve">Address {Address|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-address}
+    <t xml:space="preserve">Address {http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-address}
 </t>
   </si>
   <si>
@@ -1223,7 +1223,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="68.703125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="65.87109375" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>

<commit_message>
ci(dev): publish dev build from 10cd36323daa65b91cffa2ddd6c8fed66beef3e2 10cd36323daa65b91cffa2ddd6c8fed66beef3e2
</commit_message>
<xml_diff>
--- a/dev/StructureDefinition-ph-core-location.xlsx
+++ b/dev/StructureDefinition-ph-core-location.xlsx
@@ -9,11 +9,14 @@
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AL$62</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1392" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2144" uniqueCount="352">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-25T03:54:03+00:00</t>
+    <t>2026-04-01T03:21:07+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -617,6 +620,185 @@
     <t>.code</t>
   </si>
   <si>
+    <t>Location.type.id</t>
+  </si>
+  <si>
+    <t>Unique id for inter-element referencing</t>
+  </si>
+  <si>
+    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
+  </si>
+  <si>
+    <t>Element.id</t>
+  </si>
+  <si>
+    <t>Location.type.extension</t>
+  </si>
+  <si>
+    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value:url}
+</t>
+  </si>
+  <si>
+    <t>Extensions are always sliced by (at least) url</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>Element.extension</t>
+  </si>
+  <si>
+    <t>Location.type.coding</t>
+  </si>
+  <si>
+    <t>Code defined by a terminology system</t>
+  </si>
+  <si>
+    <t>A reference to a code defined by a terminology system.</t>
+  </si>
+  <si>
+    <t>Codes may be defined very casually in enumerations, or code lists, up to very formal definitions such as SNOMED CT - see the HL7 v3 Core Principles for more information.  Ordering of codings is undefined and SHALL NOT be used to infer meaning. Generally, at most only one of the coding values will be labeled as UserSelected = true.</t>
+  </si>
+  <si>
+    <t>Allows for alternative encodings within a code system, and translations to other code systems.</t>
+  </si>
+  <si>
+    <t>CodeableConcept.coding</t>
+  </si>
+  <si>
+    <t>union(., ./translation)</t>
+  </si>
+  <si>
+    <t>Location.type.coding.id</t>
+  </si>
+  <si>
+    <t>Location.type.coding.extension</t>
+  </si>
+  <si>
+    <t>Location.type.coding.system</t>
+  </si>
+  <si>
+    <t>Identity of the terminology system</t>
+  </si>
+  <si>
+    <t>The identification of the code system that defines the meaning of the symbol in the code.</t>
+  </si>
+  <si>
+    <t>The URI may be an OID (urn:oid:...) or a UUID (urn:uuid:...).  OIDs and UUIDs SHALL be references to the HL7 OID registry. Otherwise, the URI should come from HL7's list of FHIR defined special URIs or it should reference to some definition that establishes the system clearly and unambiguously.</t>
+  </si>
+  <si>
+    <t>Need to be unambiguous about the source of the definition of the symbol.</t>
+  </si>
+  <si>
+    <t>Coding.system</t>
+  </si>
+  <si>
+    <t>./codeSystem</t>
+  </si>
+  <si>
+    <t>Location.type.coding.version</t>
+  </si>
+  <si>
+    <t>Version of the system - if relevant</t>
+  </si>
+  <si>
+    <t>The version of the code system which was used when choosing this code. Note that a well-maintained code system does not need the version reported, because the meaning of codes is consistent across versions. However this cannot consistently be assured, and when the meaning is not guaranteed to be consistent, the version SHOULD be exchanged.</t>
+  </si>
+  <si>
+    <t>Where the terminology does not clearly define what string should be used to identify code system versions, the recommendation is to use the date (expressed in FHIR date format) on which that version was officially published as the version date.</t>
+  </si>
+  <si>
+    <t>Coding.version</t>
+  </si>
+  <si>
+    <t>./codeSystemVersion</t>
+  </si>
+  <si>
+    <t>Location.type.coding.code</t>
+  </si>
+  <si>
+    <t>Symbol in syntax defined by the system</t>
+  </si>
+  <si>
+    <t>A symbol in syntax defined by the system. The symbol may be a predefined code or an expression in a syntax defined by the coding system (e.g. post-coordination).</t>
+  </si>
+  <si>
+    <t>Need to refer to a particular code in the system.</t>
+  </si>
+  <si>
+    <t>Coding.code</t>
+  </si>
+  <si>
+    <t>./code</t>
+  </si>
+  <si>
+    <t>Location.type.coding.display</t>
+  </si>
+  <si>
+    <t>Representation defined by the system</t>
+  </si>
+  <si>
+    <t>A representation of the meaning of the code in the system, following the rules of the system.</t>
+  </si>
+  <si>
+    <t>Need to be able to carry a human-readable meaning of the code for readers that do not know  the system.</t>
+  </si>
+  <si>
+    <t>Coding.display</t>
+  </si>
+  <si>
+    <t>CV.displayName</t>
+  </si>
+  <si>
+    <t>Location.type.coding.userSelected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">boolean
+</t>
+  </si>
+  <si>
+    <t>If this coding was chosen directly by the user</t>
+  </si>
+  <si>
+    <t>Indicates that this coding was chosen by a user directly - e.g. off a pick list of available items (codes or displays).</t>
+  </si>
+  <si>
+    <t>Amongst a set of alternatives, a directly chosen code is the most appropriate starting point for new translations. There is some ambiguity about what exactly 'directly chosen' implies, and trading partner agreement may be needed to clarify the use of this element and its consequences more completely.</t>
+  </si>
+  <si>
+    <t>This has been identified as a clinical safety criterium - that this exact system/code pair was chosen explicitly, rather than inferred by the system based on some rules or language processing.</t>
+  </si>
+  <si>
+    <t>Coding.userSelected</t>
+  </si>
+  <si>
+    <t>CD.codingRationale</t>
+  </si>
+  <si>
+    <t>Location.type.text</t>
+  </si>
+  <si>
+    <t>Plain text representation of the concept</t>
+  </si>
+  <si>
+    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
+  </si>
+  <si>
+    <t>Very often the text is the same as a displayName of one of the codings.</t>
+  </si>
+  <si>
+    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
+  </si>
+  <si>
+    <t>CodeableConcept.text</t>
+  </si>
+  <si>
+    <t>./originalText[mediaType/code="text/plain"]/data</t>
+  </si>
+  <si>
     <t>Location.telecom</t>
   </si>
   <si>
@@ -679,6 +861,39 @@
     <t>.playingEntity [classCode=PLC].code</t>
   </si>
   <si>
+    <t>Location.physicalType.id</t>
+  </si>
+  <si>
+    <t>Location.physicalType.extension</t>
+  </si>
+  <si>
+    <t>Location.physicalType.coding</t>
+  </si>
+  <si>
+    <t>Location.physicalType.coding.id</t>
+  </si>
+  <si>
+    <t>Location.physicalType.coding.extension</t>
+  </si>
+  <si>
+    <t>Location.physicalType.coding.system</t>
+  </si>
+  <si>
+    <t>Location.physicalType.coding.version</t>
+  </si>
+  <si>
+    <t>Location.physicalType.coding.code</t>
+  </si>
+  <si>
+    <t>Location.physicalType.coding.display</t>
+  </si>
+  <si>
+    <t>Location.physicalType.coding.userSelected</t>
+  </si>
+  <si>
+    <t>Location.physicalType.text</t>
+  </si>
+  <si>
     <t>Location.position</t>
   </si>
   <si>
@@ -701,22 +916,7 @@
     <t>Location.position.id</t>
   </si>
   <si>
-    <t>Unique id for inter-element referencing</t>
-  </si>
-  <si>
-    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
-  </si>
-  <si>
-    <t>Element.id</t>
-  </si>
-  <si>
     <t>Location.position.extension</t>
-  </si>
-  <si>
-    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
-  </si>
-  <si>
-    <t>Element.extension</t>
   </si>
   <si>
     <t>Location.position.modifierExtension</t>
@@ -852,10 +1052,6 @@
   </si>
   <si>
     <t>Location.hoursOfOperation.allDay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">boolean
-</t>
   </si>
   <si>
     <t>The Location is open all day</t>
@@ -1037,6 +1233,21 @@
       <alignment vertical="top" wrapText="true"/>
     </xf>
   </cellXfs>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor indexed="22"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color indexed="22"/>
+        <i val="true"/>
+      </font>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -1210,7 +1421,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AL40"/>
+  <dimension ref="A1:AL62"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="36.84765625" customWidth="true" bestFit="true"/>
@@ -1241,7 +1452,7 @@
     <col min="26" max="26" width="58.125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="32" max="32" width="32.84765625" customWidth="true" bestFit="true" hidden="true"/>
@@ -1368,7 +1579,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" hidden="true">
       <c r="A2" t="s" s="2">
         <v>30</v>
       </c>
@@ -1474,7 +1685,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" hidden="true">
       <c r="A3" t="s" s="2">
         <v>83</v>
       </c>
@@ -1582,7 +1793,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" hidden="true">
       <c r="A4" t="s" s="2">
         <v>91</v>
       </c>
@@ -1688,7 +1899,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" hidden="true">
       <c r="A5" t="s" s="2">
         <v>97</v>
       </c>
@@ -1796,7 +2007,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" hidden="true">
       <c r="A6" t="s" s="2">
         <v>103</v>
       </c>
@@ -1904,7 +2115,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" hidden="true">
       <c r="A7" t="s" s="2">
         <v>112</v>
       </c>
@@ -2012,7 +2223,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" hidden="true">
       <c r="A8" t="s" s="2">
         <v>120</v>
       </c>
@@ -2120,7 +2331,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" hidden="true">
       <c r="A9" t="s" s="2">
         <v>128</v>
       </c>
@@ -2228,7 +2439,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" hidden="true">
       <c r="A10" t="s" s="2">
         <v>136</v>
       </c>
@@ -2338,7 +2549,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" hidden="true">
       <c r="A11" t="s" s="2">
         <v>141</v>
       </c>
@@ -2446,7 +2657,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" hidden="true">
       <c r="A12" t="s" s="2">
         <v>148</v>
       </c>
@@ -2552,7 +2763,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
         <v>156</v>
       </c>
@@ -2658,7 +2869,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
         <v>163</v>
       </c>
@@ -2766,7 +2977,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
         <v>169</v>
       </c>
@@ -2876,7 +3087,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
         <v>174</v>
       </c>
@@ -2984,7 +3195,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
         <v>179</v>
       </c>
@@ -3113,7 +3324,7 @@
         <v>77</v>
       </c>
       <c r="H18" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="I18" t="s" s="2">
         <v>75</v>
@@ -3200,7 +3411,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
         <v>194</v>
       </c>
@@ -3216,7 +3427,7 @@
         <v>76</v>
       </c>
       <c r="G19" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H19" t="s" s="2">
         <v>75</v>
@@ -3228,13 +3439,13 @@
         <v>75</v>
       </c>
       <c r="K19" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="L19" t="s" s="2">
         <v>195</v>
       </c>
-      <c r="L19" t="s" s="2">
+      <c r="M19" t="s" s="2">
         <v>196</v>
-      </c>
-      <c r="M19" t="s" s="2">
-        <v>197</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -3285,44 +3496,44 @@
         <v>75</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH19" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="AI19" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="AK19" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="AL19" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" hidden="true">
+      <c r="A20" t="s" s="2">
         <v>198</v>
       </c>
-      <c r="AL19" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s" s="2">
-        <v>199</v>
-      </c>
       <c r="B20" t="s" s="2">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
-        <v>75</v>
+        <v>129</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G20" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H20" t="s" s="2">
         <v>75</v>
@@ -3334,20 +3545,18 @@
         <v>75</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>201</v>
+        <v>131</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="N20" t="s" s="2">
-        <v>203</v>
-      </c>
-      <c r="O20" t="s" s="2">
-        <v>204</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
         <v>75</v>
       </c>
@@ -3383,34 +3592,34 @@
         <v>75</v>
       </c>
       <c r="AB20" t="s" s="2">
-        <v>75</v>
+        <v>200</v>
       </c>
       <c r="AC20" t="s" s="2">
-        <v>75</v>
+        <v>201</v>
       </c>
       <c r="AD20" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AE20" t="s" s="2">
-        <v>75</v>
+        <v>202</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH20" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AI20" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>96</v>
+        <v>135</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>205</v>
+        <v>162</v>
       </c>
       <c r="AL20" t="s" s="2">
         <v>75</v>
@@ -3418,10 +3627,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3432,10 +3641,10 @@
         <v>76</v>
       </c>
       <c r="G21" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H21" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="I21" t="s" s="2">
         <v>75</v>
@@ -3444,17 +3653,19 @@
         <v>85</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>188</v>
+        <v>157</v>
       </c>
       <c r="L21" t="s" s="2">
+        <v>205</v>
+      </c>
+      <c r="M21" t="s" s="2">
+        <v>206</v>
+      </c>
+      <c r="N21" t="s" s="2">
         <v>207</v>
       </c>
-      <c r="M21" t="s" s="2">
+      <c r="O21" t="s" s="2">
         <v>208</v>
-      </c>
-      <c r="N21" s="2"/>
-      <c r="O21" t="s" s="2">
-        <v>209</v>
       </c>
       <c r="P21" t="s" s="2">
         <v>75</v>
@@ -3479,13 +3690,13 @@
         <v>75</v>
       </c>
       <c r="X21" t="s" s="2">
-        <v>210</v>
+        <v>75</v>
       </c>
       <c r="Y21" t="s" s="2">
-        <v>211</v>
+        <v>75</v>
       </c>
       <c r="Z21" t="s" s="2">
-        <v>212</v>
+        <v>75</v>
       </c>
       <c r="AA21" t="s" s="2">
         <v>75</v>
@@ -3503,13 +3714,13 @@
         <v>75</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH21" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AI21" t="s" s="2">
         <v>75</v>
@@ -3518,18 +3729,18 @@
         <v>96</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>186</v>
+        <v>75</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3552,18 +3763,16 @@
         <v>75</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>215</v>
+        <v>164</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>216</v>
+        <v>195</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>217</v>
+        <v>196</v>
       </c>
       <c r="N22" s="2"/>
-      <c r="O22" t="s" s="2">
-        <v>218</v>
-      </c>
+      <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
         <v>75</v>
       </c>
@@ -3611,7 +3820,7 @@
         <v>75</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>214</v>
+        <v>197</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>76</v>
@@ -3623,32 +3832,32 @@
         <v>75</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>219</v>
+        <v>162</v>
       </c>
       <c r="AL22" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>75</v>
+        <v>129</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G23" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H23" t="s" s="2">
         <v>75</v>
@@ -3660,15 +3869,17 @@
         <v>75</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>164</v>
+        <v>130</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>221</v>
+        <v>131</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>222</v>
-      </c>
-      <c r="N23" s="2"/>
+        <v>199</v>
+      </c>
+      <c r="N23" t="s" s="2">
+        <v>133</v>
+      </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>75</v>
@@ -3705,31 +3916,31 @@
         <v>75</v>
       </c>
       <c r="AB23" t="s" s="2">
-        <v>75</v>
+        <v>200</v>
       </c>
       <c r="AC23" t="s" s="2">
-        <v>75</v>
+        <v>201</v>
       </c>
       <c r="AD23" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AE23" t="s" s="2">
-        <v>75</v>
+        <v>202</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>223</v>
+        <v>203</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH23" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AI23" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ23" t="s" s="2">
-        <v>75</v>
+        <v>135</v>
       </c>
       <c r="AK23" t="s" s="2">
         <v>162</v>
@@ -3738,23 +3949,23 @@
         <v>75</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
-        <v>129</v>
+        <v>75</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G24" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H24" t="s" s="2">
         <v>75</v>
@@ -3763,21 +3974,23 @@
         <v>75</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>130</v>
+        <v>98</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>131</v>
+        <v>214</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>133</v>
-      </c>
-      <c r="O24" s="2"/>
+        <v>216</v>
+      </c>
+      <c r="O24" t="s" s="2">
+        <v>217</v>
+      </c>
       <c r="P24" t="s" s="2">
         <v>75</v>
       </c>
@@ -3825,69 +4038,67 @@
         <v>75</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH24" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="AI24" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ24" t="s" s="2">
-        <v>135</v>
+        <v>96</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>162</v>
+        <v>219</v>
       </c>
       <c r="AL24" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>228</v>
+        <v>75</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>75</v>
       </c>
       <c r="I25" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="J25" t="s" s="2">
         <v>85</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>130</v>
+        <v>164</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>133</v>
-      </c>
-      <c r="O25" t="s" s="2">
-        <v>139</v>
-      </c>
+        <v>223</v>
+      </c>
+      <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
         <v>75</v>
       </c>
@@ -3935,22 +4146,22 @@
         <v>75</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ25" t="s" s="2">
-        <v>135</v>
+        <v>96</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>127</v>
+        <v>225</v>
       </c>
       <c r="AL25" t="s" s="2">
         <v>75</v>
@@ -3958,10 +4169,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -3969,31 +4180,33 @@
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="G26" t="s" s="2">
         <v>84</v>
       </c>
       <c r="H26" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="I26" t="s" s="2">
         <v>75</v>
       </c>
       <c r="J26" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>233</v>
+        <v>104</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
+      <c r="O26" t="s" s="2">
+        <v>229</v>
+      </c>
       <c r="P26" t="s" s="2">
         <v>75</v>
       </c>
@@ -4041,10 +4254,10 @@
         <v>75</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="AG26" t="s" s="2">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="AH26" t="s" s="2">
         <v>84</v>
@@ -4056,18 +4269,18 @@
         <v>96</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="AL26" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4075,7 +4288,7 @@
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="G27" t="s" s="2">
         <v>84</v>
@@ -4087,19 +4300,21 @@
         <v>75</v>
       </c>
       <c r="J27" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="K27" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="L27" t="s" s="2">
         <v>233</v>
       </c>
-      <c r="L27" t="s" s="2">
-        <v>238</v>
-      </c>
       <c r="M27" t="s" s="2">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="N27" s="2"/>
-      <c r="O27" s="2"/>
+      <c r="O27" t="s" s="2">
+        <v>235</v>
+      </c>
       <c r="P27" t="s" s="2">
         <v>75</v>
       </c>
@@ -4147,10 +4362,10 @@
         <v>75</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="AG27" t="s" s="2">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="AH27" t="s" s="2">
         <v>84</v>
@@ -4162,18 +4377,18 @@
         <v>96</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="AL27" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4193,19 +4408,23 @@
         <v>75</v>
       </c>
       <c r="J28" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="L28" t="s" s="2">
+        <v>240</v>
+      </c>
+      <c r="M28" t="s" s="2">
         <v>241</v>
       </c>
-      <c r="M28" t="s" s="2">
+      <c r="N28" t="s" s="2">
         <v>242</v>
       </c>
-      <c r="N28" s="2"/>
-      <c r="O28" s="2"/>
+      <c r="O28" t="s" s="2">
+        <v>243</v>
+      </c>
       <c r="P28" t="s" s="2">
         <v>75</v>
       </c>
@@ -4253,7 +4472,7 @@
         <v>75</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>76</v>
@@ -4268,18 +4487,18 @@
         <v>96</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="AL28" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4302,19 +4521,19 @@
         <v>85</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>244</v>
+        <v>164</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="O29" t="s" s="2">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="P29" t="s" s="2">
         <v>75</v>
@@ -4363,7 +4582,7 @@
         <v>75</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>76</v>
@@ -4378,18 +4597,18 @@
         <v>96</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AL29" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4400,7 +4619,7 @@
         <v>76</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>75</v>
@@ -4412,18 +4631,16 @@
         <v>75</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="N30" s="2"/>
-      <c r="O30" t="s" s="2">
-        <v>254</v>
-      </c>
+      <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>75</v>
       </c>
@@ -4471,13 +4688,13 @@
         <v>75</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AI30" t="s" s="2">
         <v>75</v>
@@ -4486,18 +4703,18 @@
         <v>96</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="AL30" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4508,7 +4725,7 @@
         <v>76</v>
       </c>
       <c r="G31" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H31" t="s" s="2">
         <v>75</v>
@@ -4520,18 +4737,20 @@
         <v>75</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>215</v>
+        <v>259</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="N31" t="s" s="2">
-        <v>259</v>
-      </c>
-      <c r="O31" s="2"/>
+        <v>262</v>
+      </c>
+      <c r="O31" t="s" s="2">
+        <v>263</v>
+      </c>
       <c r="P31" t="s" s="2">
         <v>75</v>
       </c>
@@ -4579,13 +4798,13 @@
         <v>75</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="AI31" t="s" s="2">
         <v>75</v>
@@ -4594,7 +4813,7 @@
         <v>96</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="AL31" t="s" s="2">
         <v>75</v>
@@ -4602,10 +4821,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -4619,25 +4838,27 @@
         <v>84</v>
       </c>
       <c r="H32" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="I32" t="s" s="2">
         <v>75</v>
       </c>
       <c r="J32" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>221</v>
+        <v>266</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>222</v>
+        <v>267</v>
       </c>
       <c r="N32" s="2"/>
-      <c r="O32" s="2"/>
+      <c r="O32" t="s" s="2">
+        <v>268</v>
+      </c>
       <c r="P32" t="s" s="2">
         <v>75</v>
       </c>
@@ -4661,13 +4882,13 @@
         <v>75</v>
       </c>
       <c r="X32" t="s" s="2">
-        <v>75</v>
+        <v>269</v>
       </c>
       <c r="Y32" t="s" s="2">
-        <v>75</v>
+        <v>270</v>
       </c>
       <c r="Z32" t="s" s="2">
-        <v>75</v>
+        <v>271</v>
       </c>
       <c r="AA32" t="s" s="2">
         <v>75</v>
@@ -4685,7 +4906,7 @@
         <v>75</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>223</v>
+        <v>265</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>76</v>
@@ -4697,32 +4918,32 @@
         <v>75</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>162</v>
+        <v>272</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>75</v>
+        <v>186</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>262</v>
+        <v>273</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>262</v>
+        <v>273</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>129</v>
+        <v>75</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>75</v>
@@ -4734,17 +4955,15 @@
         <v>75</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>130</v>
+        <v>164</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>131</v>
+        <v>195</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>225</v>
-      </c>
-      <c r="N33" t="s" s="2">
-        <v>133</v>
-      </c>
+        <v>196</v>
+      </c>
+      <c r="N33" s="2"/>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
         <v>75</v>
@@ -4793,19 +5012,19 @@
         <v>75</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>226</v>
+        <v>197</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ33" t="s" s="2">
-        <v>135</v>
+        <v>75</v>
       </c>
       <c r="AK33" t="s" s="2">
         <v>162</v>
@@ -4814,16 +5033,16 @@
         <v>75</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>263</v>
+        <v>274</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>263</v>
+        <v>274</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>228</v>
+        <v>129</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
@@ -4836,26 +5055,24 @@
         <v>75</v>
       </c>
       <c r="I34" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="J34" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="K34" t="s" s="2">
         <v>130</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>229</v>
+        <v>131</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>230</v>
+        <v>199</v>
       </c>
       <c r="N34" t="s" s="2">
         <v>133</v>
       </c>
-      <c r="O34" t="s" s="2">
-        <v>139</v>
-      </c>
+      <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
         <v>75</v>
       </c>
@@ -4891,19 +5108,19 @@
         <v>75</v>
       </c>
       <c r="AB34" t="s" s="2">
-        <v>75</v>
+        <v>200</v>
       </c>
       <c r="AC34" t="s" s="2">
-        <v>75</v>
+        <v>201</v>
       </c>
       <c r="AD34" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AE34" t="s" s="2">
-        <v>75</v>
+        <v>202</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>231</v>
+        <v>203</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>76</v>
@@ -4918,7 +5135,7 @@
         <v>135</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="AL34" t="s" s="2">
         <v>75</v>
@@ -4926,10 +5143,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>264</v>
+        <v>275</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>264</v>
+        <v>275</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -4943,25 +5160,29 @@
         <v>77</v>
       </c>
       <c r="H35" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="I35" t="s" s="2">
         <v>75</v>
       </c>
       <c r="J35" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>104</v>
+        <v>157</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>265</v>
+        <v>205</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>266</v>
-      </c>
-      <c r="N35" s="2"/>
-      <c r="O35" s="2"/>
+        <v>206</v>
+      </c>
+      <c r="N35" t="s" s="2">
+        <v>207</v>
+      </c>
+      <c r="O35" t="s" s="2">
+        <v>208</v>
+      </c>
       <c r="P35" t="s" s="2">
         <v>75</v>
       </c>
@@ -4985,13 +5206,13 @@
         <v>75</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>151</v>
+        <v>75</v>
       </c>
       <c r="Y35" t="s" s="2">
-        <v>267</v>
+        <v>75</v>
       </c>
       <c r="Z35" t="s" s="2">
-        <v>268</v>
+        <v>75</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>75</v>
@@ -5009,7 +5230,7 @@
         <v>75</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>264</v>
+        <v>209</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>76</v>
@@ -5024,18 +5245,18 @@
         <v>96</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>260</v>
+        <v>210</v>
       </c>
       <c r="AL35" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5058,13 +5279,13 @@
         <v>75</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>270</v>
+        <v>164</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>271</v>
+        <v>195</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>272</v>
+        <v>196</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -5115,7 +5336,7 @@
         <v>75</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>269</v>
+        <v>197</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>76</v>
@@ -5127,32 +5348,32 @@
         <v>75</v>
       </c>
       <c r="AJ36" t="s" s="2">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>260</v>
+        <v>162</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>75</v>
+        <v>129</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>75</v>
@@ -5164,15 +5385,17 @@
         <v>75</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>274</v>
+        <v>130</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>275</v>
+        <v>131</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>276</v>
-      </c>
-      <c r="N37" s="2"/>
+        <v>199</v>
+      </c>
+      <c r="N37" t="s" s="2">
+        <v>133</v>
+      </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
         <v>75</v>
@@ -5209,45 +5432,45 @@
         <v>75</v>
       </c>
       <c r="AB37" t="s" s="2">
-        <v>75</v>
+        <v>200</v>
       </c>
       <c r="AC37" t="s" s="2">
-        <v>75</v>
+        <v>201</v>
       </c>
       <c r="AD37" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AE37" t="s" s="2">
-        <v>75</v>
+        <v>202</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>273</v>
+        <v>203</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AI37" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>96</v>
+        <v>135</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>260</v>
+        <v>162</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5267,19 +5490,23 @@
         <v>75</v>
       </c>
       <c r="J38" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>274</v>
+        <v>98</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>278</v>
+        <v>214</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>279</v>
-      </c>
-      <c r="N38" s="2"/>
-      <c r="O38" s="2"/>
+        <v>215</v>
+      </c>
+      <c r="N38" t="s" s="2">
+        <v>216</v>
+      </c>
+      <c r="O38" t="s" s="2">
+        <v>217</v>
+      </c>
       <c r="P38" t="s" s="2">
         <v>75</v>
       </c>
@@ -5327,7 +5554,7 @@
         <v>75</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>277</v>
+        <v>218</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>76</v>
@@ -5342,18 +5569,18 @@
         <v>96</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>260</v>
+        <v>219</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5373,18 +5600,20 @@
         <v>75</v>
       </c>
       <c r="J39" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="K39" t="s" s="2">
         <v>164</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>281</v>
+        <v>221</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>282</v>
-      </c>
-      <c r="N39" s="2"/>
+        <v>222</v>
+      </c>
+      <c r="N39" t="s" s="2">
+        <v>223</v>
+      </c>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>75</v>
@@ -5433,7 +5662,7 @@
         <v>75</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>280</v>
+        <v>224</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>76</v>
@@ -5448,7 +5677,7 @@
         <v>96</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>162</v>
+        <v>225</v>
       </c>
       <c r="AL39" t="s" s="2">
         <v>75</v>
@@ -5456,10 +5685,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5470,29 +5699,29 @@
         <v>76</v>
       </c>
       <c r="G40" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H40" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="I40" t="s" s="2">
         <v>75</v>
       </c>
       <c r="J40" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>284</v>
+        <v>104</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>285</v>
+        <v>227</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>286</v>
+        <v>228</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" t="s" s="2">
-        <v>287</v>
+        <v>229</v>
       </c>
       <c r="P40" t="s" s="2">
         <v>75</v>
@@ -5541,13 +5770,13 @@
         <v>75</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>283</v>
+        <v>230</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH40" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="AI40" t="s" s="2">
         <v>75</v>
@@ -5556,13 +5785,2397 @@
         <v>96</v>
       </c>
       <c r="AK40" t="s" s="2">
+        <v>231</v>
+      </c>
+      <c r="AL40" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="41" hidden="true">
+      <c r="A41" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="B41" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="C41" s="2"/>
+      <c r="D41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E41" s="2"/>
+      <c r="F41" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G41" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J41" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="K41" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="L41" t="s" s="2">
+        <v>233</v>
+      </c>
+      <c r="M41" t="s" s="2">
+        <v>234</v>
+      </c>
+      <c r="N41" s="2"/>
+      <c r="O41" t="s" s="2">
+        <v>235</v>
+      </c>
+      <c r="P41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q41" s="2"/>
+      <c r="R41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF41" t="s" s="2">
+        <v>236</v>
+      </c>
+      <c r="AG41" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH41" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI41" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ41" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK41" t="s" s="2">
+        <v>237</v>
+      </c>
+      <c r="AL41" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="42" hidden="true">
+      <c r="A42" t="s" s="2">
+        <v>282</v>
+      </c>
+      <c r="B42" t="s" s="2">
+        <v>282</v>
+      </c>
+      <c r="C42" s="2"/>
+      <c r="D42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E42" s="2"/>
+      <c r="F42" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G42" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J42" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="K42" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="L42" t="s" s="2">
+        <v>240</v>
+      </c>
+      <c r="M42" t="s" s="2">
+        <v>241</v>
+      </c>
+      <c r="N42" t="s" s="2">
+        <v>242</v>
+      </c>
+      <c r="O42" t="s" s="2">
+        <v>243</v>
+      </c>
+      <c r="P42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q42" s="2"/>
+      <c r="R42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF42" t="s" s="2">
+        <v>244</v>
+      </c>
+      <c r="AG42" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH42" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ42" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK42" t="s" s="2">
+        <v>245</v>
+      </c>
+      <c r="AL42" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="43" hidden="true">
+      <c r="A43" t="s" s="2">
+        <v>283</v>
+      </c>
+      <c r="B43" t="s" s="2">
+        <v>283</v>
+      </c>
+      <c r="C43" s="2"/>
+      <c r="D43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E43" s="2"/>
+      <c r="F43" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G43" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J43" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="K43" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="L43" t="s" s="2">
+        <v>247</v>
+      </c>
+      <c r="M43" t="s" s="2">
+        <v>248</v>
+      </c>
+      <c r="N43" t="s" s="2">
+        <v>249</v>
+      </c>
+      <c r="O43" t="s" s="2">
+        <v>250</v>
+      </c>
+      <c r="P43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q43" s="2"/>
+      <c r="R43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF43" t="s" s="2">
+        <v>251</v>
+      </c>
+      <c r="AG43" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH43" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ43" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK43" t="s" s="2">
+        <v>252</v>
+      </c>
+      <c r="AL43" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="44" hidden="true">
+      <c r="A44" t="s" s="2">
+        <v>284</v>
+      </c>
+      <c r="B44" t="s" s="2">
+        <v>284</v>
+      </c>
+      <c r="C44" s="2"/>
+      <c r="D44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E44" s="2"/>
+      <c r="F44" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G44" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K44" t="s" s="2">
+        <v>285</v>
+      </c>
+      <c r="L44" t="s" s="2">
+        <v>286</v>
+      </c>
+      <c r="M44" t="s" s="2">
+        <v>287</v>
+      </c>
+      <c r="N44" s="2"/>
+      <c r="O44" t="s" s="2">
+        <v>288</v>
+      </c>
+      <c r="P44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q44" s="2"/>
+      <c r="R44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF44" t="s" s="2">
+        <v>284</v>
+      </c>
+      <c r="AG44" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH44" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ44" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK44" t="s" s="2">
+        <v>289</v>
+      </c>
+      <c r="AL44" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="45" hidden="true">
+      <c r="A45" t="s" s="2">
+        <v>290</v>
+      </c>
+      <c r="B45" t="s" s="2">
+        <v>290</v>
+      </c>
+      <c r="C45" s="2"/>
+      <c r="D45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E45" s="2"/>
+      <c r="F45" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G45" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K45" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="L45" t="s" s="2">
+        <v>195</v>
+      </c>
+      <c r="M45" t="s" s="2">
+        <v>196</v>
+      </c>
+      <c r="N45" s="2"/>
+      <c r="O45" s="2"/>
+      <c r="P45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q45" s="2"/>
+      <c r="R45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF45" t="s" s="2">
+        <v>197</v>
+      </c>
+      <c r="AG45" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH45" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AK45" t="s" s="2">
         <v>162</v>
       </c>
-      <c r="AL40" t="s" s="2">
+      <c r="AL45" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="46" hidden="true">
+      <c r="A46" t="s" s="2">
+        <v>291</v>
+      </c>
+      <c r="B46" t="s" s="2">
+        <v>291</v>
+      </c>
+      <c r="C46" s="2"/>
+      <c r="D46" t="s" s="2">
+        <v>129</v>
+      </c>
+      <c r="E46" s="2"/>
+      <c r="F46" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K46" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="L46" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="M46" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="N46" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="O46" s="2"/>
+      <c r="P46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q46" s="2"/>
+      <c r="R46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF46" t="s" s="2">
+        <v>203</v>
+      </c>
+      <c r="AG46" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AI46" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ46" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="AK46" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="AL46" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="47" hidden="true">
+      <c r="A47" t="s" s="2">
+        <v>292</v>
+      </c>
+      <c r="B47" t="s" s="2">
+        <v>292</v>
+      </c>
+      <c r="C47" s="2"/>
+      <c r="D47" t="s" s="2">
+        <v>293</v>
+      </c>
+      <c r="E47" s="2"/>
+      <c r="F47" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I47" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="J47" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="K47" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="L47" t="s" s="2">
+        <v>294</v>
+      </c>
+      <c r="M47" t="s" s="2">
+        <v>295</v>
+      </c>
+      <c r="N47" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="O47" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="P47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q47" s="2"/>
+      <c r="R47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF47" t="s" s="2">
+        <v>296</v>
+      </c>
+      <c r="AG47" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AI47" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ47" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="AK47" t="s" s="2">
+        <v>127</v>
+      </c>
+      <c r="AL47" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="48" hidden="true">
+      <c r="A48" t="s" s="2">
+        <v>297</v>
+      </c>
+      <c r="B48" t="s" s="2">
+        <v>297</v>
+      </c>
+      <c r="C48" s="2"/>
+      <c r="D48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E48" s="2"/>
+      <c r="F48" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="G48" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K48" t="s" s="2">
+        <v>298</v>
+      </c>
+      <c r="L48" t="s" s="2">
+        <v>299</v>
+      </c>
+      <c r="M48" t="s" s="2">
+        <v>300</v>
+      </c>
+      <c r="N48" s="2"/>
+      <c r="O48" s="2"/>
+      <c r="P48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q48" s="2"/>
+      <c r="R48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF48" t="s" s="2">
+        <v>297</v>
+      </c>
+      <c r="AG48" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AH48" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI48" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ48" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK48" t="s" s="2">
+        <v>301</v>
+      </c>
+      <c r="AL48" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="49" hidden="true">
+      <c r="A49" t="s" s="2">
+        <v>302</v>
+      </c>
+      <c r="B49" t="s" s="2">
+        <v>302</v>
+      </c>
+      <c r="C49" s="2"/>
+      <c r="D49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E49" s="2"/>
+      <c r="F49" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="G49" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K49" t="s" s="2">
+        <v>298</v>
+      </c>
+      <c r="L49" t="s" s="2">
+        <v>303</v>
+      </c>
+      <c r="M49" t="s" s="2">
+        <v>304</v>
+      </c>
+      <c r="N49" s="2"/>
+      <c r="O49" s="2"/>
+      <c r="P49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q49" s="2"/>
+      <c r="R49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF49" t="s" s="2">
+        <v>302</v>
+      </c>
+      <c r="AG49" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AH49" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ49" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK49" t="s" s="2">
+        <v>301</v>
+      </c>
+      <c r="AL49" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="50" hidden="true">
+      <c r="A50" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="B50" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="C50" s="2"/>
+      <c r="D50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E50" s="2"/>
+      <c r="F50" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G50" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K50" t="s" s="2">
+        <v>298</v>
+      </c>
+      <c r="L50" t="s" s="2">
+        <v>306</v>
+      </c>
+      <c r="M50" t="s" s="2">
+        <v>307</v>
+      </c>
+      <c r="N50" s="2"/>
+      <c r="O50" s="2"/>
+      <c r="P50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q50" s="2"/>
+      <c r="R50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF50" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="AG50" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH50" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI50" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ50" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK50" t="s" s="2">
+        <v>301</v>
+      </c>
+      <c r="AL50" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="51" hidden="true">
+      <c r="A51" t="s" s="2">
+        <v>308</v>
+      </c>
+      <c r="B51" t="s" s="2">
+        <v>308</v>
+      </c>
+      <c r="C51" s="2"/>
+      <c r="D51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E51" s="2"/>
+      <c r="F51" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G51" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J51" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="K51" t="s" s="2">
+        <v>309</v>
+      </c>
+      <c r="L51" t="s" s="2">
+        <v>310</v>
+      </c>
+      <c r="M51" t="s" s="2">
+        <v>311</v>
+      </c>
+      <c r="N51" t="s" s="2">
+        <v>312</v>
+      </c>
+      <c r="O51" t="s" s="2">
+        <v>313</v>
+      </c>
+      <c r="P51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q51" s="2"/>
+      <c r="R51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF51" t="s" s="2">
+        <v>308</v>
+      </c>
+      <c r="AG51" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH51" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI51" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ51" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK51" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="AL51" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="52" hidden="true">
+      <c r="A52" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="B52" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="C52" s="2"/>
+      <c r="D52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E52" s="2"/>
+      <c r="F52" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G52" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K52" t="s" s="2">
+        <v>316</v>
+      </c>
+      <c r="L52" t="s" s="2">
+        <v>317</v>
+      </c>
+      <c r="M52" t="s" s="2">
+        <v>318</v>
+      </c>
+      <c r="N52" s="2"/>
+      <c r="O52" t="s" s="2">
+        <v>319</v>
+      </c>
+      <c r="P52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q52" s="2"/>
+      <c r="R52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF52" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="AG52" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH52" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI52" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ52" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK52" t="s" s="2">
+        <v>320</v>
+      </c>
+      <c r="AL52" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="53" hidden="true">
+      <c r="A53" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="B53" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="C53" s="2"/>
+      <c r="D53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E53" s="2"/>
+      <c r="F53" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K53" t="s" s="2">
+        <v>285</v>
+      </c>
+      <c r="L53" t="s" s="2">
+        <v>322</v>
+      </c>
+      <c r="M53" t="s" s="2">
+        <v>323</v>
+      </c>
+      <c r="N53" t="s" s="2">
+        <v>324</v>
+      </c>
+      <c r="O53" s="2"/>
+      <c r="P53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q53" s="2"/>
+      <c r="R53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF53" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="AG53" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AI53" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ53" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK53" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="AL53" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="54" hidden="true">
+      <c r="A54" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="B54" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="C54" s="2"/>
+      <c r="D54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E54" s="2"/>
+      <c r="F54" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G54" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K54" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="L54" t="s" s="2">
+        <v>195</v>
+      </c>
+      <c r="M54" t="s" s="2">
+        <v>196</v>
+      </c>
+      <c r="N54" s="2"/>
+      <c r="O54" s="2"/>
+      <c r="P54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q54" s="2"/>
+      <c r="R54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF54" t="s" s="2">
+        <v>197</v>
+      </c>
+      <c r="AG54" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH54" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ54" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AK54" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="AL54" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="55" hidden="true">
+      <c r="A55" t="s" s="2">
+        <v>327</v>
+      </c>
+      <c r="B55" t="s" s="2">
+        <v>327</v>
+      </c>
+      <c r="C55" s="2"/>
+      <c r="D55" t="s" s="2">
+        <v>129</v>
+      </c>
+      <c r="E55" s="2"/>
+      <c r="F55" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G55" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K55" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="L55" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="M55" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="N55" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="O55" s="2"/>
+      <c r="P55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q55" s="2"/>
+      <c r="R55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF55" t="s" s="2">
+        <v>203</v>
+      </c>
+      <c r="AG55" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH55" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AI55" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ55" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="AK55" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="AL55" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="56" hidden="true">
+      <c r="A56" t="s" s="2">
+        <v>328</v>
+      </c>
+      <c r="B56" t="s" s="2">
+        <v>328</v>
+      </c>
+      <c r="C56" s="2"/>
+      <c r="D56" t="s" s="2">
+        <v>293</v>
+      </c>
+      <c r="E56" s="2"/>
+      <c r="F56" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G56" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I56" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="J56" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="K56" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="L56" t="s" s="2">
+        <v>294</v>
+      </c>
+      <c r="M56" t="s" s="2">
+        <v>295</v>
+      </c>
+      <c r="N56" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="O56" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="P56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q56" s="2"/>
+      <c r="R56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF56" t="s" s="2">
+        <v>296</v>
+      </c>
+      <c r="AG56" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH56" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AI56" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ56" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="AK56" t="s" s="2">
+        <v>127</v>
+      </c>
+      <c r="AL56" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="57" hidden="true">
+      <c r="A57" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="B57" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="C57" s="2"/>
+      <c r="D57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E57" s="2"/>
+      <c r="F57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G57" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K57" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="L57" t="s" s="2">
+        <v>330</v>
+      </c>
+      <c r="M57" t="s" s="2">
+        <v>331</v>
+      </c>
+      <c r="N57" s="2"/>
+      <c r="O57" s="2"/>
+      <c r="P57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q57" s="2"/>
+      <c r="R57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X57" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="Y57" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="Z57" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="AA57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF57" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="AG57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH57" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AI57" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ57" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK57" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="AL57" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="58" hidden="true">
+      <c r="A58" t="s" s="2">
+        <v>334</v>
+      </c>
+      <c r="B58" t="s" s="2">
+        <v>334</v>
+      </c>
+      <c r="C58" s="2"/>
+      <c r="D58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E58" s="2"/>
+      <c r="F58" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G58" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K58" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="L58" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="M58" t="s" s="2">
+        <v>336</v>
+      </c>
+      <c r="N58" s="2"/>
+      <c r="O58" s="2"/>
+      <c r="P58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q58" s="2"/>
+      <c r="R58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF58" t="s" s="2">
+        <v>334</v>
+      </c>
+      <c r="AG58" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH58" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI58" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ58" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK58" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="AL58" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="59" hidden="true">
+      <c r="A59" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="B59" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="C59" s="2"/>
+      <c r="D59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E59" s="2"/>
+      <c r="F59" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G59" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K59" t="s" s="2">
+        <v>338</v>
+      </c>
+      <c r="L59" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="M59" t="s" s="2">
+        <v>340</v>
+      </c>
+      <c r="N59" s="2"/>
+      <c r="O59" s="2"/>
+      <c r="P59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q59" s="2"/>
+      <c r="R59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF59" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="AG59" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH59" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI59" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ59" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK59" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="AL59" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="60" hidden="true">
+      <c r="A60" t="s" s="2">
+        <v>341</v>
+      </c>
+      <c r="B60" t="s" s="2">
+        <v>341</v>
+      </c>
+      <c r="C60" s="2"/>
+      <c r="D60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E60" s="2"/>
+      <c r="F60" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G60" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K60" t="s" s="2">
+        <v>338</v>
+      </c>
+      <c r="L60" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="M60" t="s" s="2">
+        <v>343</v>
+      </c>
+      <c r="N60" s="2"/>
+      <c r="O60" s="2"/>
+      <c r="P60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q60" s="2"/>
+      <c r="R60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF60" t="s" s="2">
+        <v>341</v>
+      </c>
+      <c r="AG60" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH60" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI60" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ60" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK60" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="AL60" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="61" hidden="true">
+      <c r="A61" t="s" s="2">
+        <v>344</v>
+      </c>
+      <c r="B61" t="s" s="2">
+        <v>344</v>
+      </c>
+      <c r="C61" s="2"/>
+      <c r="D61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E61" s="2"/>
+      <c r="F61" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G61" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K61" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="L61" t="s" s="2">
+        <v>345</v>
+      </c>
+      <c r="M61" t="s" s="2">
+        <v>346</v>
+      </c>
+      <c r="N61" s="2"/>
+      <c r="O61" s="2"/>
+      <c r="P61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q61" s="2"/>
+      <c r="R61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF61" t="s" s="2">
+        <v>344</v>
+      </c>
+      <c r="AG61" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH61" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI61" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ61" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK61" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="AL61" t="s" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="62" hidden="true">
+      <c r="A62" t="s" s="2">
+        <v>347</v>
+      </c>
+      <c r="B62" t="s" s="2">
+        <v>347</v>
+      </c>
+      <c r="C62" s="2"/>
+      <c r="D62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="E62" s="2"/>
+      <c r="F62" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G62" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K62" t="s" s="2">
+        <v>348</v>
+      </c>
+      <c r="L62" t="s" s="2">
+        <v>349</v>
+      </c>
+      <c r="M62" t="s" s="2">
+        <v>350</v>
+      </c>
+      <c r="N62" s="2"/>
+      <c r="O62" t="s" s="2">
+        <v>351</v>
+      </c>
+      <c r="P62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Q62" s="2"/>
+      <c r="R62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="S62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="T62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="U62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="V62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="W62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="X62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Y62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="Z62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AA62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AB62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AC62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AD62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AE62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AF62" t="s" s="2">
+        <v>347</v>
+      </c>
+      <c r="AG62" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH62" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AI62" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AJ62" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AK62" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="AL62" t="s" s="2">
         <v>75</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AL62">
+    <filterColumn colId="7">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+    <filterColumn colId="27">
+      <filters blank="true"/>
+    </filterColumn>
+  </autoFilter>
+  <conditionalFormatting sqref="A2:AI61">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$G2&lt;&gt;"Y"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>$Q2&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ci(dev): publish dev build from 40391d988dc18cdb145bb63fbee903c6100cc59e 40391d988dc18cdb145bb63fbee903c6100cc59e
</commit_message>
<xml_diff>
--- a/dev/StructureDefinition-ph-core-location.xlsx
+++ b/dev/StructureDefinition-ph-core-location.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AL$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AL$48</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2144" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1666" uniqueCount="311">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-06T07:53:57+00:00</t>
+    <t>2026-04-08T04:01:15+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -672,386 +672,263 @@
     <t>union(., ./translation)</t>
   </si>
   <si>
-    <t>Location.type.coding.id</t>
-  </si>
-  <si>
-    <t>Location.type.coding.extension</t>
-  </si>
-  <si>
-    <t>Location.type.coding.system</t>
-  </si>
-  <si>
-    <t>Identity of the terminology system</t>
-  </si>
-  <si>
-    <t>The identification of the code system that defines the meaning of the symbol in the code.</t>
-  </si>
-  <si>
-    <t>The URI may be an OID (urn:oid:...) or a UUID (urn:uuid:...).  OIDs and UUIDs SHALL be references to the HL7 OID registry. Otherwise, the URI should come from HL7's list of FHIR defined special URIs or it should reference to some definition that establishes the system clearly and unambiguously.</t>
-  </si>
-  <si>
-    <t>Need to be unambiguous about the source of the definition of the symbol.</t>
-  </si>
-  <si>
-    <t>Coding.system</t>
-  </si>
-  <si>
-    <t>./codeSystem</t>
-  </si>
-  <si>
-    <t>Location.type.coding.version</t>
-  </si>
-  <si>
-    <t>Version of the system - if relevant</t>
-  </si>
-  <si>
-    <t>The version of the code system which was used when choosing this code. Note that a well-maintained code system does not need the version reported, because the meaning of codes is consistent across versions. However this cannot consistently be assured, and when the meaning is not guaranteed to be consistent, the version SHOULD be exchanged.</t>
-  </si>
-  <si>
-    <t>Where the terminology does not clearly define what string should be used to identify code system versions, the recommendation is to use the date (expressed in FHIR date format) on which that version was officially published as the version date.</t>
-  </si>
-  <si>
-    <t>Coding.version</t>
-  </si>
-  <si>
-    <t>./codeSystemVersion</t>
-  </si>
-  <si>
-    <t>Location.type.coding.code</t>
-  </si>
-  <si>
-    <t>Symbol in syntax defined by the system</t>
-  </si>
-  <si>
-    <t>A symbol in syntax defined by the system. The symbol may be a predefined code or an expression in a syntax defined by the coding system (e.g. post-coordination).</t>
-  </si>
-  <si>
-    <t>Need to refer to a particular code in the system.</t>
-  </si>
-  <si>
-    <t>Coding.code</t>
-  </si>
-  <si>
-    <t>./code</t>
-  </si>
-  <si>
-    <t>Location.type.coding.display</t>
-  </si>
-  <si>
-    <t>Representation defined by the system</t>
-  </si>
-  <si>
-    <t>A representation of the meaning of the code in the system, following the rules of the system.</t>
-  </si>
-  <si>
-    <t>Need to be able to carry a human-readable meaning of the code for readers that do not know  the system.</t>
-  </si>
-  <si>
-    <t>Coding.display</t>
-  </si>
-  <si>
-    <t>CV.displayName</t>
-  </si>
-  <si>
-    <t>Location.type.coding.userSelected</t>
+    <t>Location.type.text</t>
+  </si>
+  <si>
+    <t>Plain text representation of the concept</t>
+  </si>
+  <si>
+    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
+  </si>
+  <si>
+    <t>Very often the text is the same as a displayName of one of the codings.</t>
+  </si>
+  <si>
+    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
+  </si>
+  <si>
+    <t>CodeableConcept.text</t>
+  </si>
+  <si>
+    <t>./originalText[mediaType/code="text/plain"]/data</t>
+  </si>
+  <si>
+    <t>Location.telecom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ContactPoint
+</t>
+  </si>
+  <si>
+    <t>Contact details of the location</t>
+  </si>
+  <si>
+    <t>The contact details of communication devices available at the location. This can include phone numbers, fax numbers, mobile numbers, email addresses and web sites.</t>
+  </si>
+  <si>
+    <t>.telecom</t>
+  </si>
+  <si>
+    <t>Location.address</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address {http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-address}
+</t>
+  </si>
+  <si>
+    <t>Physical location</t>
+  </si>
+  <si>
+    <t>Physical location.</t>
+  </si>
+  <si>
+    <t>Additional addresses should be recorded using another instance of the Location resource, or via the Organization.</t>
+  </si>
+  <si>
+    <t>If locations can be visited, we need to keep track of their address.</t>
+  </si>
+  <si>
+    <t>.addr</t>
+  </si>
+  <si>
+    <t>Location.physicalType</t>
+  </si>
+  <si>
+    <t>Physical form of the location</t>
+  </si>
+  <si>
+    <t>Physical form of the location, e.g. building, room, vehicle, road.</t>
+  </si>
+  <si>
+    <t>For purposes of showing relevant locations in queries, we need to categorize locations.</t>
+  </si>
+  <si>
+    <t>example</t>
+  </si>
+  <si>
+    <t>Physical form of the location.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/location-physical-type|4.0.1</t>
+  </si>
+  <si>
+    <t>.playingEntity [classCode=PLC].code</t>
+  </si>
+  <si>
+    <t>Location.physicalType.id</t>
+  </si>
+  <si>
+    <t>Location.physicalType.extension</t>
+  </si>
+  <si>
+    <t>Location.physicalType.coding</t>
+  </si>
+  <si>
+    <t>Location.physicalType.text</t>
+  </si>
+  <si>
+    <t>Location.position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BackboneElement
+</t>
+  </si>
+  <si>
+    <t>The absolute geographic location</t>
+  </si>
+  <si>
+    <t>The absolute geographic location of the Location, expressed using the WGS84 datum (This is the same co-ordinate system used in KML).</t>
+  </si>
+  <si>
+    <t>For mobile applications and automated route-finding knowing the exact location of the Location is required.</t>
+  </si>
+  <si>
+    <t>.playingEntity [classCode=PLC determinerCode=INSTANCE].positionText</t>
+  </si>
+  <si>
+    <t>Location.position.id</t>
+  </si>
+  <si>
+    <t>Location.position.extension</t>
+  </si>
+  <si>
+    <t>Location.position.modifierExtension</t>
+  </si>
+  <si>
+    <t>extensions
+user contentmodifiers</t>
+  </si>
+  <si>
+    <t>Extensions that cannot be ignored even if unrecognized</t>
+  </si>
+  <si>
+    <t>May be used to represent additional information that is not part of the basic definition of the element and that modifies the understanding of the element in which it is contained and/or the understanding of the containing element's descendants. Usually modifier elements provide negation or qualification. To make the use of extensions safe and manageable, there is a strict set of governance applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension. Applications processing a resource are required to check for modifier extensions.
+Modifier extensions SHALL NOT change the meaning of any elements on Resource or DomainResource (including cannot change the meaning of modifierExtension itself).</t>
+  </si>
+  <si>
+    <t>BackboneElement.modifierExtension</t>
+  </si>
+  <si>
+    <t>Location.position.longitude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">decimal
+</t>
+  </si>
+  <si>
+    <t>Longitude with WGS84 datum</t>
+  </si>
+  <si>
+    <t>Longitude. The value domain and the interpretation are the same as for the text of the longitude element in KML (see notes below).</t>
+  </si>
+  <si>
+    <t>(RIM Opted not to map the sub-elements of GPS location, is now an OBS)</t>
+  </si>
+  <si>
+    <t>Location.position.latitude</t>
+  </si>
+  <si>
+    <t>Latitude with WGS84 datum</t>
+  </si>
+  <si>
+    <t>Latitude. The value domain and the interpretation are the same as for the text of the latitude element in KML (see notes below).</t>
+  </si>
+  <si>
+    <t>Location.position.altitude</t>
+  </si>
+  <si>
+    <t>Altitude with WGS84 datum</t>
+  </si>
+  <si>
+    <t>Altitude. The value domain and the interpretation are the same as for the text of the altitude element in KML (see notes below).</t>
+  </si>
+  <si>
+    <t>Location.managingOrganization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-organization)
+</t>
+  </si>
+  <si>
+    <t>Organization responsible for provisioning and upkeep</t>
+  </si>
+  <si>
+    <t>The organization responsible for the provisioning and upkeep of the location.</t>
+  </si>
+  <si>
+    <t>This can also be used as the part of the organization hierarchy where this location provides services. These services can be defined through the HealthcareService resource.</t>
+  </si>
+  <si>
+    <t>Need to know who manages the location.</t>
+  </si>
+  <si>
+    <t>.scopingEntity[classCode=ORG determinerKind=INSTANCE]</t>
+  </si>
+  <si>
+    <t>Location.partOf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-location)
+</t>
+  </si>
+  <si>
+    <t>Another Location this one is physically a part of</t>
+  </si>
+  <si>
+    <t>Another Location of which this Location is physically a part of.</t>
+  </si>
+  <si>
+    <t>For purposes of location, display and identification, knowing which locations are located within other locations is important.</t>
+  </si>
+  <si>
+    <t>.inboundLink[typeCode=PART].source[classCode=SDLC]</t>
+  </si>
+  <si>
+    <t>Location.hoursOfOperation</t>
+  </si>
+  <si>
+    <t>What days/times during a week is this location usually open</t>
+  </si>
+  <si>
+    <t>What days/times during a week is this location usually open.</t>
+  </si>
+  <si>
+    <t>This type of information is commonly found published in directories and on websites informing customers when the facility is available.
+Specific services within the location may have their own hours which could be shorter (or longer) than the locations hours.</t>
+  </si>
+  <si>
+    <t>.effectiveTime</t>
+  </si>
+  <si>
+    <t>Location.hoursOfOperation.id</t>
+  </si>
+  <si>
+    <t>Location.hoursOfOperation.extension</t>
+  </si>
+  <si>
+    <t>Location.hoursOfOperation.modifierExtension</t>
+  </si>
+  <si>
+    <t>Location.hoursOfOperation.daysOfWeek</t>
+  </si>
+  <si>
+    <t>mon | tue | wed | thu | fri | sat | sun</t>
+  </si>
+  <si>
+    <t>Indicates which days of the week are available between the start and end Times.</t>
+  </si>
+  <si>
+    <t>The days of the week.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/days-of-week|4.0.1</t>
+  </si>
+  <si>
+    <t>Location.hoursOfOperation.allDay</t>
   </si>
   <si>
     <t xml:space="preserve">boolean
 </t>
-  </si>
-  <si>
-    <t>If this coding was chosen directly by the user</t>
-  </si>
-  <si>
-    <t>Indicates that this coding was chosen by a user directly - e.g. off a pick list of available items (codes or displays).</t>
-  </si>
-  <si>
-    <t>Amongst a set of alternatives, a directly chosen code is the most appropriate starting point for new translations. There is some ambiguity about what exactly 'directly chosen' implies, and trading partner agreement may be needed to clarify the use of this element and its consequences more completely.</t>
-  </si>
-  <si>
-    <t>This has been identified as a clinical safety criterium - that this exact system/code pair was chosen explicitly, rather than inferred by the system based on some rules or language processing.</t>
-  </si>
-  <si>
-    <t>Coding.userSelected</t>
-  </si>
-  <si>
-    <t>CD.codingRationale</t>
-  </si>
-  <si>
-    <t>Location.type.text</t>
-  </si>
-  <si>
-    <t>Plain text representation of the concept</t>
-  </si>
-  <si>
-    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
-  </si>
-  <si>
-    <t>Very often the text is the same as a displayName of one of the codings.</t>
-  </si>
-  <si>
-    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
-  </si>
-  <si>
-    <t>CodeableConcept.text</t>
-  </si>
-  <si>
-    <t>./originalText[mediaType/code="text/plain"]/data</t>
-  </si>
-  <si>
-    <t>Location.telecom</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ContactPoint
-</t>
-  </si>
-  <si>
-    <t>Contact details of the location</t>
-  </si>
-  <si>
-    <t>The contact details of communication devices available at the location. This can include phone numbers, fax numbers, mobile numbers, email addresses and web sites.</t>
-  </si>
-  <si>
-    <t>.telecom</t>
-  </si>
-  <si>
-    <t>Location.address</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Address {http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-address}
-</t>
-  </si>
-  <si>
-    <t>Physical location</t>
-  </si>
-  <si>
-    <t>Physical location.</t>
-  </si>
-  <si>
-    <t>Additional addresses should be recorded using another instance of the Location resource, or via the Organization.</t>
-  </si>
-  <si>
-    <t>If locations can be visited, we need to keep track of their address.</t>
-  </si>
-  <si>
-    <t>.addr</t>
-  </si>
-  <si>
-    <t>Location.physicalType</t>
-  </si>
-  <si>
-    <t>Physical form of the location</t>
-  </si>
-  <si>
-    <t>Physical form of the location, e.g. building, room, vehicle, road.</t>
-  </si>
-  <si>
-    <t>For purposes of showing relevant locations in queries, we need to categorize locations.</t>
-  </si>
-  <si>
-    <t>example</t>
-  </si>
-  <si>
-    <t>Physical form of the location.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/location-physical-type|4.0.1</t>
-  </si>
-  <si>
-    <t>.playingEntity [classCode=PLC].code</t>
-  </si>
-  <si>
-    <t>Location.physicalType.id</t>
-  </si>
-  <si>
-    <t>Location.physicalType.extension</t>
-  </si>
-  <si>
-    <t>Location.physicalType.coding</t>
-  </si>
-  <si>
-    <t>Location.physicalType.coding.id</t>
-  </si>
-  <si>
-    <t>Location.physicalType.coding.extension</t>
-  </si>
-  <si>
-    <t>Location.physicalType.coding.system</t>
-  </si>
-  <si>
-    <t>Location.physicalType.coding.version</t>
-  </si>
-  <si>
-    <t>Location.physicalType.coding.code</t>
-  </si>
-  <si>
-    <t>Location.physicalType.coding.display</t>
-  </si>
-  <si>
-    <t>Location.physicalType.coding.userSelected</t>
-  </si>
-  <si>
-    <t>Location.physicalType.text</t>
-  </si>
-  <si>
-    <t>Location.position</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BackboneElement
-</t>
-  </si>
-  <si>
-    <t>The absolute geographic location</t>
-  </si>
-  <si>
-    <t>The absolute geographic location of the Location, expressed using the WGS84 datum (This is the same co-ordinate system used in KML).</t>
-  </si>
-  <si>
-    <t>For mobile applications and automated route-finding knowing the exact location of the Location is required.</t>
-  </si>
-  <si>
-    <t>.playingEntity [classCode=PLC determinerCode=INSTANCE].positionText</t>
-  </si>
-  <si>
-    <t>Location.position.id</t>
-  </si>
-  <si>
-    <t>Location.position.extension</t>
-  </si>
-  <si>
-    <t>Location.position.modifierExtension</t>
-  </si>
-  <si>
-    <t>extensions
-user contentmodifiers</t>
-  </si>
-  <si>
-    <t>Extensions that cannot be ignored even if unrecognized</t>
-  </si>
-  <si>
-    <t>May be used to represent additional information that is not part of the basic definition of the element and that modifies the understanding of the element in which it is contained and/or the understanding of the containing element's descendants. Usually modifier elements provide negation or qualification. To make the use of extensions safe and manageable, there is a strict set of governance applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension. Applications processing a resource are required to check for modifier extensions.
-Modifier extensions SHALL NOT change the meaning of any elements on Resource or DomainResource (including cannot change the meaning of modifierExtension itself).</t>
-  </si>
-  <si>
-    <t>BackboneElement.modifierExtension</t>
-  </si>
-  <si>
-    <t>Location.position.longitude</t>
-  </si>
-  <si>
-    <t xml:space="preserve">decimal
-</t>
-  </si>
-  <si>
-    <t>Longitude with WGS84 datum</t>
-  </si>
-  <si>
-    <t>Longitude. The value domain and the interpretation are the same as for the text of the longitude element in KML (see notes below).</t>
-  </si>
-  <si>
-    <t>(RIM Opted not to map the sub-elements of GPS location, is now an OBS)</t>
-  </si>
-  <si>
-    <t>Location.position.latitude</t>
-  </si>
-  <si>
-    <t>Latitude with WGS84 datum</t>
-  </si>
-  <si>
-    <t>Latitude. The value domain and the interpretation are the same as for the text of the latitude element in KML (see notes below).</t>
-  </si>
-  <si>
-    <t>Location.position.altitude</t>
-  </si>
-  <si>
-    <t>Altitude with WGS84 datum</t>
-  </si>
-  <si>
-    <t>Altitude. The value domain and the interpretation are the same as for the text of the altitude element in KML (see notes below).</t>
-  </si>
-  <si>
-    <t>Location.managingOrganization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-organization)
-</t>
-  </si>
-  <si>
-    <t>Organization responsible for provisioning and upkeep</t>
-  </si>
-  <si>
-    <t>The organization responsible for the provisioning and upkeep of the location.</t>
-  </si>
-  <si>
-    <t>This can also be used as the part of the organization hierarchy where this location provides services. These services can be defined through the HealthcareService resource.</t>
-  </si>
-  <si>
-    <t>Need to know who manages the location.</t>
-  </si>
-  <si>
-    <t>.scopingEntity[classCode=ORG determinerKind=INSTANCE]</t>
-  </si>
-  <si>
-    <t>Location.partOf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-location)
-</t>
-  </si>
-  <si>
-    <t>Another Location this one is physically a part of</t>
-  </si>
-  <si>
-    <t>Another Location of which this Location is physically a part of.</t>
-  </si>
-  <si>
-    <t>For purposes of location, display and identification, knowing which locations are located within other locations is important.</t>
-  </si>
-  <si>
-    <t>.inboundLink[typeCode=PART].source[classCode=SDLC]</t>
-  </si>
-  <si>
-    <t>Location.hoursOfOperation</t>
-  </si>
-  <si>
-    <t>What days/times during a week is this location usually open</t>
-  </si>
-  <si>
-    <t>What days/times during a week is this location usually open.</t>
-  </si>
-  <si>
-    <t>This type of information is commonly found published in directories and on websites informing customers when the facility is available.
-Specific services within the location may have their own hours which could be shorter (or longer) than the locations hours.</t>
-  </si>
-  <si>
-    <t>.effectiveTime</t>
-  </si>
-  <si>
-    <t>Location.hoursOfOperation.id</t>
-  </si>
-  <si>
-    <t>Location.hoursOfOperation.extension</t>
-  </si>
-  <si>
-    <t>Location.hoursOfOperation.modifierExtension</t>
-  </si>
-  <si>
-    <t>Location.hoursOfOperation.daysOfWeek</t>
-  </si>
-  <si>
-    <t>mon | tue | wed | thu | fri | sat | sun</t>
-  </si>
-  <si>
-    <t>Indicates which days of the week are available between the start and end Times.</t>
-  </si>
-  <si>
-    <t>The days of the week.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/days-of-week|4.0.1</t>
-  </si>
-  <si>
-    <t>Location.hoursOfOperation.allDay</t>
   </si>
   <si>
     <t>The Location is open all day</t>
@@ -1421,7 +1298,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AL62"/>
+  <dimension ref="A1:AL48"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="36.84765625" customWidth="true" bestFit="true"/>
@@ -3735,7 +3612,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22" hidden="true">
+    <row r="22">
       <c r="A22" t="s" s="2">
         <v>211</v>
       </c>
@@ -3754,25 +3631,29 @@
         <v>84</v>
       </c>
       <c r="H22" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="I22" t="s" s="2">
         <v>75</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="K22" t="s" s="2">
         <v>164</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>195</v>
+        <v>212</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>196</v>
-      </c>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2"/>
+        <v>213</v>
+      </c>
+      <c r="N22" t="s" s="2">
+        <v>214</v>
+      </c>
+      <c r="O22" t="s" s="2">
+        <v>215</v>
+      </c>
       <c r="P22" t="s" s="2">
         <v>75</v>
       </c>
@@ -3820,7 +3701,7 @@
         <v>75</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>76</v>
@@ -3832,10 +3713,10 @@
         <v>75</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>162</v>
+        <v>217</v>
       </c>
       <c r="AL22" t="s" s="2">
         <v>75</v>
@@ -3843,14 +3724,14 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>129</v>
+        <v>75</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
@@ -3869,17 +3750,15 @@
         <v>75</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>130</v>
+        <v>219</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>131</v>
+        <v>220</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>199</v>
-      </c>
-      <c r="N23" t="s" s="2">
-        <v>133</v>
-      </c>
+        <v>221</v>
+      </c>
+      <c r="N23" s="2"/>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>75</v>
@@ -3916,19 +3795,19 @@
         <v>75</v>
       </c>
       <c r="AB23" t="s" s="2">
-        <v>200</v>
+        <v>75</v>
       </c>
       <c r="AC23" t="s" s="2">
-        <v>201</v>
+        <v>75</v>
       </c>
       <c r="AD23" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AE23" t="s" s="2">
-        <v>202</v>
+        <v>75</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>76</v>
@@ -3940,10 +3819,10 @@
         <v>75</v>
       </c>
       <c r="AJ23" t="s" s="2">
-        <v>135</v>
+        <v>96</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>162</v>
+        <v>222</v>
       </c>
       <c r="AL23" t="s" s="2">
         <v>75</v>
@@ -3951,10 +3830,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3974,22 +3853,22 @@
         <v>75</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>98</v>
+        <v>224</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>216</v>
+        <v>227</v>
       </c>
       <c r="O24" t="s" s="2">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>75</v>
@@ -4038,7 +3917,7 @@
         <v>75</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>76</v>
@@ -4053,18 +3932,18 @@
         <v>96</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="AL24" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="25" hidden="true">
+    <row r="25">
       <c r="A25" t="s" s="2">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4078,7 +3957,7 @@
         <v>84</v>
       </c>
       <c r="H25" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="I25" t="s" s="2">
         <v>75</v>
@@ -4087,18 +3966,18 @@
         <v>85</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>222</v>
-      </c>
-      <c r="N25" t="s" s="2">
-        <v>223</v>
-      </c>
-      <c r="O25" s="2"/>
+        <v>232</v>
+      </c>
+      <c r="N25" s="2"/>
+      <c r="O25" t="s" s="2">
+        <v>233</v>
+      </c>
       <c r="P25" t="s" s="2">
         <v>75</v>
       </c>
@@ -4122,13 +4001,13 @@
         <v>75</v>
       </c>
       <c r="X25" t="s" s="2">
-        <v>75</v>
+        <v>234</v>
       </c>
       <c r="Y25" t="s" s="2">
-        <v>75</v>
+        <v>235</v>
       </c>
       <c r="Z25" t="s" s="2">
-        <v>75</v>
+        <v>236</v>
       </c>
       <c r="AA25" t="s" s="2">
         <v>75</v>
@@ -4146,7 +4025,7 @@
         <v>75</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>76</v>
@@ -4161,18 +4040,18 @@
         <v>96</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4186,27 +4065,25 @@
         <v>84</v>
       </c>
       <c r="H26" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="I26" t="s" s="2">
         <v>75</v>
       </c>
       <c r="J26" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>104</v>
+        <v>164</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>227</v>
+        <v>195</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>228</v>
+        <v>196</v>
       </c>
       <c r="N26" s="2"/>
-      <c r="O26" t="s" s="2">
-        <v>229</v>
-      </c>
+      <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
         <v>75</v>
       </c>
@@ -4254,7 +4131,7 @@
         <v>75</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>230</v>
+        <v>197</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>76</v>
@@ -4266,10 +4143,10 @@
         <v>75</v>
       </c>
       <c r="AJ26" t="s" s="2">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>231</v>
+        <v>162</v>
       </c>
       <c r="AL26" t="s" s="2">
         <v>75</v>
@@ -4277,21 +4154,21 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
-        <v>75</v>
+        <v>129</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G27" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H27" t="s" s="2">
         <v>75</v>
@@ -4300,21 +4177,21 @@
         <v>75</v>
       </c>
       <c r="J27" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>164</v>
+        <v>130</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>233</v>
+        <v>131</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>234</v>
-      </c>
-      <c r="N27" s="2"/>
-      <c r="O27" t="s" s="2">
-        <v>235</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="N27" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
         <v>75</v>
       </c>
@@ -4350,45 +4227,45 @@
         <v>75</v>
       </c>
       <c r="AB27" t="s" s="2">
-        <v>75</v>
+        <v>200</v>
       </c>
       <c r="AC27" t="s" s="2">
-        <v>75</v>
+        <v>201</v>
       </c>
       <c r="AD27" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AE27" t="s" s="2">
-        <v>75</v>
+        <v>202</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>236</v>
+        <v>203</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH27" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AI27" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>96</v>
+        <v>135</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>237</v>
+        <v>162</v>
       </c>
       <c r="AL27" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="28" hidden="true">
+    <row r="28">
       <c r="A28" t="s" s="2">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4399,10 +4276,10 @@
         <v>76</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H28" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="I28" t="s" s="2">
         <v>75</v>
@@ -4411,19 +4288,19 @@
         <v>85</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>239</v>
+        <v>157</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>241</v>
+        <v>206</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>242</v>
+        <v>207</v>
       </c>
       <c r="O28" t="s" s="2">
-        <v>243</v>
+        <v>208</v>
       </c>
       <c r="P28" t="s" s="2">
         <v>75</v>
@@ -4472,13 +4349,13 @@
         <v>75</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>244</v>
+        <v>209</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AI28" t="s" s="2">
         <v>75</v>
@@ -4487,18 +4364,18 @@
         <v>96</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>245</v>
+        <v>210</v>
       </c>
       <c r="AL28" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="29" hidden="true">
+    <row r="29">
       <c r="A29" t="s" s="2">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4512,7 +4389,7 @@
         <v>84</v>
       </c>
       <c r="H29" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="I29" t="s" s="2">
         <v>75</v>
@@ -4524,16 +4401,16 @@
         <v>164</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>247</v>
+        <v>212</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>248</v>
+        <v>213</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>249</v>
+        <v>214</v>
       </c>
       <c r="O29" t="s" s="2">
-        <v>250</v>
+        <v>215</v>
       </c>
       <c r="P29" t="s" s="2">
         <v>75</v>
@@ -4582,7 +4459,7 @@
         <v>75</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>251</v>
+        <v>216</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>76</v>
@@ -4597,7 +4474,7 @@
         <v>96</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>252</v>
+        <v>217</v>
       </c>
       <c r="AL29" t="s" s="2">
         <v>75</v>
@@ -4605,10 +4482,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4619,7 +4496,7 @@
         <v>76</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>75</v>
@@ -4631,16 +4508,18 @@
         <v>75</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>255</v>
+        <v>244</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="N30" s="2"/>
-      <c r="O30" s="2"/>
+      <c r="O30" t="s" s="2">
+        <v>246</v>
+      </c>
       <c r="P30" t="s" s="2">
         <v>75</v>
       </c>
@@ -4688,13 +4567,13 @@
         <v>75</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="AI30" t="s" s="2">
         <v>75</v>
@@ -4703,7 +4582,7 @@
         <v>96</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="AL30" t="s" s="2">
         <v>75</v>
@@ -4711,10 +4590,10 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4737,20 +4616,16 @@
         <v>75</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>259</v>
+        <v>164</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>260</v>
+        <v>195</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>261</v>
-      </c>
-      <c r="N31" t="s" s="2">
-        <v>262</v>
-      </c>
-      <c r="O31" t="s" s="2">
-        <v>263</v>
-      </c>
+        <v>196</v>
+      </c>
+      <c r="N31" s="2"/>
+      <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
         <v>75</v>
       </c>
@@ -4798,7 +4673,7 @@
         <v>75</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>258</v>
+        <v>197</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>76</v>
@@ -4810,55 +4685,55 @@
         <v>75</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>264</v>
+        <v>162</v>
       </c>
       <c r="AL31" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>265</v>
+        <v>249</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>265</v>
+        <v>249</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>75</v>
+        <v>129</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G32" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H32" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="I32" t="s" s="2">
         <v>75</v>
       </c>
       <c r="J32" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>188</v>
+        <v>130</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>266</v>
+        <v>131</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>267</v>
-      </c>
-      <c r="N32" s="2"/>
-      <c r="O32" t="s" s="2">
-        <v>268</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="N32" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
         <v>75</v>
       </c>
@@ -4882,13 +4757,13 @@
         <v>75</v>
       </c>
       <c r="X32" t="s" s="2">
-        <v>269</v>
+        <v>75</v>
       </c>
       <c r="Y32" t="s" s="2">
-        <v>270</v>
+        <v>75</v>
       </c>
       <c r="Z32" t="s" s="2">
-        <v>271</v>
+        <v>75</v>
       </c>
       <c r="AA32" t="s" s="2">
         <v>75</v>
@@ -4906,65 +4781,69 @@
         <v>75</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>265</v>
+        <v>203</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH32" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AI32" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>96</v>
+        <v>135</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>272</v>
+        <v>162</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>186</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>273</v>
+        <v>250</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>273</v>
+        <v>250</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>75</v>
+        <v>251</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>75</v>
       </c>
       <c r="I33" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="J33" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>164</v>
+        <v>130</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>195</v>
+        <v>252</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>196</v>
-      </c>
-      <c r="N33" s="2"/>
-      <c r="O33" s="2"/>
+        <v>253</v>
+      </c>
+      <c r="N33" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="O33" t="s" s="2">
+        <v>139</v>
+      </c>
       <c r="P33" t="s" s="2">
         <v>75</v>
       </c>
@@ -5012,22 +4891,22 @@
         <v>75</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>197</v>
+        <v>254</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ33" t="s" s="2">
-        <v>75</v>
+        <v>135</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>162</v>
+        <v>127</v>
       </c>
       <c r="AL33" t="s" s="2">
         <v>75</v>
@@ -5035,21 +4914,21 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>274</v>
+        <v>255</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>274</v>
+        <v>255</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>129</v>
+        <v>75</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H34" t="s" s="2">
         <v>75</v>
@@ -5061,17 +4940,15 @@
         <v>75</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>130</v>
+        <v>256</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>131</v>
+        <v>257</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>199</v>
-      </c>
-      <c r="N34" t="s" s="2">
-        <v>133</v>
-      </c>
+        <v>258</v>
+      </c>
+      <c r="N34" s="2"/>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
         <v>75</v>
@@ -5108,45 +4985,45 @@
         <v>75</v>
       </c>
       <c r="AB34" t="s" s="2">
-        <v>200</v>
+        <v>75</v>
       </c>
       <c r="AC34" t="s" s="2">
-        <v>201</v>
+        <v>75</v>
       </c>
       <c r="AD34" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AE34" t="s" s="2">
-        <v>202</v>
+        <v>75</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>203</v>
+        <v>255</v>
       </c>
       <c r="AG34" t="s" s="2">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="AH34" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="AI34" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>135</v>
+        <v>96</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>162</v>
+        <v>259</v>
       </c>
       <c r="AL34" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5154,35 +5031,31 @@
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G35" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H35" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="I35" t="s" s="2">
         <v>75</v>
       </c>
       <c r="J35" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>157</v>
+        <v>256</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>205</v>
+        <v>261</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>206</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>207</v>
-      </c>
-      <c r="O35" t="s" s="2">
-        <v>208</v>
-      </c>
+        <v>262</v>
+      </c>
+      <c r="N35" s="2"/>
+      <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
         <v>75</v>
       </c>
@@ -5230,13 +5103,13 @@
         <v>75</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>209</v>
+        <v>260</v>
       </c>
       <c r="AG35" t="s" s="2">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="AH35" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="AI35" t="s" s="2">
         <v>75</v>
@@ -5245,7 +5118,7 @@
         <v>96</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>210</v>
+        <v>259</v>
       </c>
       <c r="AL35" t="s" s="2">
         <v>75</v>
@@ -5253,10 +5126,10 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>276</v>
+        <v>263</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>276</v>
+        <v>263</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5279,13 +5152,13 @@
         <v>75</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>164</v>
+        <v>256</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>195</v>
+        <v>264</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>196</v>
+        <v>265</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -5336,7 +5209,7 @@
         <v>75</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>197</v>
+        <v>263</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>76</v>
@@ -5348,10 +5221,10 @@
         <v>75</v>
       </c>
       <c r="AJ36" t="s" s="2">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>162</v>
+        <v>259</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>75</v>
@@ -5359,21 +5232,21 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>129</v>
+        <v>75</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>75</v>
@@ -5382,21 +5255,23 @@
         <v>75</v>
       </c>
       <c r="J37" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>130</v>
+        <v>267</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>131</v>
+        <v>268</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>199</v>
+        <v>269</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>133</v>
-      </c>
-      <c r="O37" s="2"/>
+        <v>270</v>
+      </c>
+      <c r="O37" t="s" s="2">
+        <v>271</v>
+      </c>
       <c r="P37" t="s" s="2">
         <v>75</v>
       </c>
@@ -5432,34 +5307,34 @@
         <v>75</v>
       </c>
       <c r="AB37" t="s" s="2">
-        <v>200</v>
+        <v>75</v>
       </c>
       <c r="AC37" t="s" s="2">
-        <v>201</v>
+        <v>75</v>
       </c>
       <c r="AD37" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AE37" t="s" s="2">
-        <v>202</v>
+        <v>75</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>203</v>
+        <v>266</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="AI37" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>135</v>
+        <v>96</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>162</v>
+        <v>272</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>75</v>
@@ -5467,10 +5342,10 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5490,22 +5365,20 @@
         <v>75</v>
       </c>
       <c r="J38" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>98</v>
+        <v>274</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>214</v>
+        <v>275</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>215</v>
-      </c>
-      <c r="N38" t="s" s="2">
-        <v>216</v>
-      </c>
+        <v>276</v>
+      </c>
+      <c r="N38" s="2"/>
       <c r="O38" t="s" s="2">
-        <v>217</v>
+        <v>277</v>
       </c>
       <c r="P38" t="s" s="2">
         <v>75</v>
@@ -5554,7 +5427,7 @@
         <v>75</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>218</v>
+        <v>273</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>76</v>
@@ -5569,7 +5442,7 @@
         <v>96</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>219</v>
+        <v>278</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>75</v>
@@ -5591,7 +5464,7 @@
         <v>76</v>
       </c>
       <c r="G39" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H39" t="s" s="2">
         <v>75</v>
@@ -5600,19 +5473,19 @@
         <v>75</v>
       </c>
       <c r="J39" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>164</v>
+        <v>243</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>221</v>
+        <v>280</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>222</v>
+        <v>281</v>
       </c>
       <c r="N39" t="s" s="2">
-        <v>223</v>
+        <v>282</v>
       </c>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
@@ -5662,13 +5535,13 @@
         <v>75</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>224</v>
+        <v>279</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH39" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AI39" t="s" s="2">
         <v>75</v>
@@ -5677,18 +5550,18 @@
         <v>96</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>225</v>
+        <v>283</v>
       </c>
       <c r="AL39" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5702,27 +5575,25 @@
         <v>84</v>
       </c>
       <c r="H40" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="I40" t="s" s="2">
         <v>75</v>
       </c>
       <c r="J40" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>104</v>
+        <v>164</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>227</v>
+        <v>195</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>228</v>
+        <v>196</v>
       </c>
       <c r="N40" s="2"/>
-      <c r="O40" t="s" s="2">
-        <v>229</v>
-      </c>
+      <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
         <v>75</v>
       </c>
@@ -5770,7 +5641,7 @@
         <v>75</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>230</v>
+        <v>197</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>76</v>
@@ -5782,10 +5653,10 @@
         <v>75</v>
       </c>
       <c r="AJ40" t="s" s="2">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>231</v>
+        <v>162</v>
       </c>
       <c r="AL40" t="s" s="2">
         <v>75</v>
@@ -5793,21 +5664,21 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
-        <v>75</v>
+        <v>129</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G41" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H41" t="s" s="2">
         <v>75</v>
@@ -5816,21 +5687,21 @@
         <v>75</v>
       </c>
       <c r="J41" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>164</v>
+        <v>130</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>233</v>
+        <v>131</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>234</v>
-      </c>
-      <c r="N41" s="2"/>
-      <c r="O41" t="s" s="2">
-        <v>235</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="N41" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
         <v>75</v>
       </c>
@@ -5878,22 +5749,22 @@
         <v>75</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>236</v>
+        <v>203</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH41" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AI41" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>96</v>
+        <v>135</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>237</v>
+        <v>162</v>
       </c>
       <c r="AL41" t="s" s="2">
         <v>75</v>
@@ -5901,45 +5772,45 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>75</v>
+        <v>251</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G42" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H42" t="s" s="2">
         <v>75</v>
       </c>
       <c r="I42" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="J42" t="s" s="2">
         <v>85</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>239</v>
+        <v>130</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="N42" t="s" s="2">
-        <v>242</v>
+        <v>133</v>
       </c>
       <c r="O42" t="s" s="2">
-        <v>243</v>
+        <v>139</v>
       </c>
       <c r="P42" t="s" s="2">
         <v>75</v>
@@ -5988,22 +5859,22 @@
         <v>75</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH42" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AI42" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>96</v>
+        <v>135</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>245</v>
+        <v>127</v>
       </c>
       <c r="AL42" t="s" s="2">
         <v>75</v>
@@ -6011,10 +5882,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6025,7 +5896,7 @@
         <v>76</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H43" t="s" s="2">
         <v>75</v>
@@ -6034,23 +5905,19 @@
         <v>75</v>
       </c>
       <c r="J43" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>164</v>
+        <v>104</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>247</v>
+        <v>288</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>248</v>
-      </c>
-      <c r="N43" t="s" s="2">
-        <v>249</v>
-      </c>
-      <c r="O43" t="s" s="2">
-        <v>250</v>
-      </c>
+        <v>289</v>
+      </c>
+      <c r="N43" s="2"/>
+      <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
         <v>75</v>
       </c>
@@ -6074,13 +5941,13 @@
         <v>75</v>
       </c>
       <c r="X43" t="s" s="2">
-        <v>75</v>
+        <v>151</v>
       </c>
       <c r="Y43" t="s" s="2">
-        <v>75</v>
+        <v>290</v>
       </c>
       <c r="Z43" t="s" s="2">
-        <v>75</v>
+        <v>291</v>
       </c>
       <c r="AA43" t="s" s="2">
         <v>75</v>
@@ -6098,13 +5965,13 @@
         <v>75</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>251</v>
+        <v>287</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH43" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AI43" t="s" s="2">
         <v>75</v>
@@ -6113,7 +5980,7 @@
         <v>96</v>
       </c>
       <c r="AK43" t="s" s="2">
-        <v>252</v>
+        <v>283</v>
       </c>
       <c r="AL43" t="s" s="2">
         <v>75</v>
@@ -6121,10 +5988,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6147,18 +6014,16 @@
         <v>75</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="N44" s="2"/>
-      <c r="O44" t="s" s="2">
-        <v>288</v>
-      </c>
+      <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
         <v>75</v>
       </c>
@@ -6206,7 +6071,7 @@
         <v>75</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>76</v>
@@ -6221,7 +6086,7 @@
         <v>96</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="AL44" t="s" s="2">
         <v>75</v>
@@ -6229,10 +6094,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6255,13 +6120,13 @@
         <v>75</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>164</v>
+        <v>297</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>195</v>
+        <v>298</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>196</v>
+        <v>299</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -6312,7 +6177,7 @@
         <v>75</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>197</v>
+        <v>296</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>76</v>
@@ -6324,10 +6189,10 @@
         <v>75</v>
       </c>
       <c r="AJ45" t="s" s="2">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>162</v>
+        <v>283</v>
       </c>
       <c r="AL45" t="s" s="2">
         <v>75</v>
@@ -6335,21 +6200,21 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
-        <v>129</v>
+        <v>75</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G46" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H46" t="s" s="2">
         <v>75</v>
@@ -6361,17 +6226,15 @@
         <v>75</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>130</v>
+        <v>297</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>131</v>
+        <v>301</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>199</v>
-      </c>
-      <c r="N46" t="s" s="2">
-        <v>133</v>
-      </c>
+        <v>302</v>
+      </c>
+      <c r="N46" s="2"/>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
         <v>75</v>
@@ -6420,22 +6283,22 @@
         <v>75</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>203</v>
+        <v>300</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH46" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="AI46" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>135</v>
+        <v>96</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>162</v>
+        <v>283</v>
       </c>
       <c r="AL46" t="s" s="2">
         <v>75</v>
@@ -6443,46 +6306,42 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>292</v>
+        <v>303</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>292</v>
+        <v>303</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
-        <v>293</v>
+        <v>75</v>
       </c>
       <c r="E47" s="2"/>
       <c r="F47" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G47" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H47" t="s" s="2">
         <v>75</v>
       </c>
       <c r="I47" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="J47" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>130</v>
+        <v>164</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>294</v>
+        <v>304</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>295</v>
-      </c>
-      <c r="N47" t="s" s="2">
-        <v>133</v>
-      </c>
-      <c r="O47" t="s" s="2">
-        <v>139</v>
-      </c>
+        <v>305</v>
+      </c>
+      <c r="N47" s="2"/>
+      <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
         <v>75</v>
       </c>
@@ -6530,22 +6389,22 @@
         <v>75</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH47" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="AI47" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AJ47" t="s" s="2">
-        <v>135</v>
+        <v>96</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="AL47" t="s" s="2">
         <v>75</v>
@@ -6553,10 +6412,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -6564,10 +6423,10 @@
       </c>
       <c r="E48" s="2"/>
       <c r="F48" t="s" s="2">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="G48" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H48" t="s" s="2">
         <v>75</v>
@@ -6579,16 +6438,18 @@
         <v>75</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>298</v>
+        <v>307</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>300</v>
+        <v>309</v>
       </c>
       <c r="N48" s="2"/>
-      <c r="O48" s="2"/>
+      <c r="O48" t="s" s="2">
+        <v>310</v>
+      </c>
       <c r="P48" t="s" s="2">
         <v>75</v>
       </c>
@@ -6636,13 +6497,13 @@
         <v>75</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="AG48" t="s" s="2">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="AH48" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AI48" t="s" s="2">
         <v>75</v>
@@ -6651,1514 +6512,14 @@
         <v>96</v>
       </c>
       <c r="AK48" t="s" s="2">
-        <v>301</v>
+        <v>162</v>
       </c>
       <c r="AL48" t="s" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="49" hidden="true">
-      <c r="A49" t="s" s="2">
-        <v>302</v>
-      </c>
-      <c r="B49" t="s" s="2">
-        <v>302</v>
-      </c>
-      <c r="C49" s="2"/>
-      <c r="D49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E49" s="2"/>
-      <c r="F49" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="G49" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K49" t="s" s="2">
-        <v>298</v>
-      </c>
-      <c r="L49" t="s" s="2">
-        <v>303</v>
-      </c>
-      <c r="M49" t="s" s="2">
-        <v>304</v>
-      </c>
-      <c r="N49" s="2"/>
-      <c r="O49" s="2"/>
-      <c r="P49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q49" s="2"/>
-      <c r="R49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF49" t="s" s="2">
-        <v>302</v>
-      </c>
-      <c r="AG49" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH49" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI49" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ49" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AK49" t="s" s="2">
-        <v>301</v>
-      </c>
-      <c r="AL49" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="50" hidden="true">
-      <c r="A50" t="s" s="2">
-        <v>305</v>
-      </c>
-      <c r="B50" t="s" s="2">
-        <v>305</v>
-      </c>
-      <c r="C50" s="2"/>
-      <c r="D50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E50" s="2"/>
-      <c r="F50" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G50" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K50" t="s" s="2">
-        <v>298</v>
-      </c>
-      <c r="L50" t="s" s="2">
-        <v>306</v>
-      </c>
-      <c r="M50" t="s" s="2">
-        <v>307</v>
-      </c>
-      <c r="N50" s="2"/>
-      <c r="O50" s="2"/>
-      <c r="P50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q50" s="2"/>
-      <c r="R50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF50" t="s" s="2">
-        <v>305</v>
-      </c>
-      <c r="AG50" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH50" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI50" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ50" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AK50" t="s" s="2">
-        <v>301</v>
-      </c>
-      <c r="AL50" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="51" hidden="true">
-      <c r="A51" t="s" s="2">
-        <v>308</v>
-      </c>
-      <c r="B51" t="s" s="2">
-        <v>308</v>
-      </c>
-      <c r="C51" s="2"/>
-      <c r="D51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E51" s="2"/>
-      <c r="F51" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G51" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J51" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="K51" t="s" s="2">
-        <v>309</v>
-      </c>
-      <c r="L51" t="s" s="2">
-        <v>310</v>
-      </c>
-      <c r="M51" t="s" s="2">
-        <v>311</v>
-      </c>
-      <c r="N51" t="s" s="2">
-        <v>312</v>
-      </c>
-      <c r="O51" t="s" s="2">
-        <v>313</v>
-      </c>
-      <c r="P51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q51" s="2"/>
-      <c r="R51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF51" t="s" s="2">
-        <v>308</v>
-      </c>
-      <c r="AG51" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH51" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI51" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ51" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AK51" t="s" s="2">
-        <v>314</v>
-      </c>
-      <c r="AL51" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="52" hidden="true">
-      <c r="A52" t="s" s="2">
-        <v>315</v>
-      </c>
-      <c r="B52" t="s" s="2">
-        <v>315</v>
-      </c>
-      <c r="C52" s="2"/>
-      <c r="D52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E52" s="2"/>
-      <c r="F52" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G52" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K52" t="s" s="2">
-        <v>316</v>
-      </c>
-      <c r="L52" t="s" s="2">
-        <v>317</v>
-      </c>
-      <c r="M52" t="s" s="2">
-        <v>318</v>
-      </c>
-      <c r="N52" s="2"/>
-      <c r="O52" t="s" s="2">
-        <v>319</v>
-      </c>
-      <c r="P52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q52" s="2"/>
-      <c r="R52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF52" t="s" s="2">
-        <v>315</v>
-      </c>
-      <c r="AG52" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH52" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI52" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ52" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AK52" t="s" s="2">
-        <v>320</v>
-      </c>
-      <c r="AL52" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="53" hidden="true">
-      <c r="A53" t="s" s="2">
-        <v>321</v>
-      </c>
-      <c r="B53" t="s" s="2">
-        <v>321</v>
-      </c>
-      <c r="C53" s="2"/>
-      <c r="D53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E53" s="2"/>
-      <c r="F53" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="H53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K53" t="s" s="2">
-        <v>285</v>
-      </c>
-      <c r="L53" t="s" s="2">
-        <v>322</v>
-      </c>
-      <c r="M53" t="s" s="2">
-        <v>323</v>
-      </c>
-      <c r="N53" t="s" s="2">
-        <v>324</v>
-      </c>
-      <c r="O53" s="2"/>
-      <c r="P53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q53" s="2"/>
-      <c r="R53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF53" t="s" s="2">
-        <v>321</v>
-      </c>
-      <c r="AG53" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AI53" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ53" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AK53" t="s" s="2">
-        <v>325</v>
-      </c>
-      <c r="AL53" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="54" hidden="true">
-      <c r="A54" t="s" s="2">
-        <v>326</v>
-      </c>
-      <c r="B54" t="s" s="2">
-        <v>326</v>
-      </c>
-      <c r="C54" s="2"/>
-      <c r="D54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E54" s="2"/>
-      <c r="F54" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G54" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K54" t="s" s="2">
-        <v>164</v>
-      </c>
-      <c r="L54" t="s" s="2">
-        <v>195</v>
-      </c>
-      <c r="M54" t="s" s="2">
-        <v>196</v>
-      </c>
-      <c r="N54" s="2"/>
-      <c r="O54" s="2"/>
-      <c r="P54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q54" s="2"/>
-      <c r="R54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF54" t="s" s="2">
-        <v>197</v>
-      </c>
-      <c r="AG54" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH54" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ54" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK54" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AL54" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="55" hidden="true">
-      <c r="A55" t="s" s="2">
-        <v>327</v>
-      </c>
-      <c r="B55" t="s" s="2">
-        <v>327</v>
-      </c>
-      <c r="C55" s="2"/>
-      <c r="D55" t="s" s="2">
-        <v>129</v>
-      </c>
-      <c r="E55" s="2"/>
-      <c r="F55" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="H55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K55" t="s" s="2">
-        <v>130</v>
-      </c>
-      <c r="L55" t="s" s="2">
-        <v>131</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>199</v>
-      </c>
-      <c r="N55" t="s" s="2">
-        <v>133</v>
-      </c>
-      <c r="O55" s="2"/>
-      <c r="P55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q55" s="2"/>
-      <c r="R55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF55" t="s" s="2">
-        <v>203</v>
-      </c>
-      <c r="AG55" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AI55" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ55" t="s" s="2">
-        <v>135</v>
-      </c>
-      <c r="AK55" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AL55" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="56" hidden="true">
-      <c r="A56" t="s" s="2">
-        <v>328</v>
-      </c>
-      <c r="B56" t="s" s="2">
-        <v>328</v>
-      </c>
-      <c r="C56" s="2"/>
-      <c r="D56" t="s" s="2">
-        <v>293</v>
-      </c>
-      <c r="E56" s="2"/>
-      <c r="F56" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="H56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I56" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="J56" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="K56" t="s" s="2">
-        <v>130</v>
-      </c>
-      <c r="L56" t="s" s="2">
-        <v>294</v>
-      </c>
-      <c r="M56" t="s" s="2">
-        <v>295</v>
-      </c>
-      <c r="N56" t="s" s="2">
-        <v>133</v>
-      </c>
-      <c r="O56" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="P56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q56" s="2"/>
-      <c r="R56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF56" t="s" s="2">
-        <v>296</v>
-      </c>
-      <c r="AG56" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AI56" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ56" t="s" s="2">
-        <v>135</v>
-      </c>
-      <c r="AK56" t="s" s="2">
-        <v>127</v>
-      </c>
-      <c r="AL56" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="57" hidden="true">
-      <c r="A57" t="s" s="2">
-        <v>329</v>
-      </c>
-      <c r="B57" t="s" s="2">
-        <v>329</v>
-      </c>
-      <c r="C57" s="2"/>
-      <c r="D57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E57" s="2"/>
-      <c r="F57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="H57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K57" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="L57" t="s" s="2">
-        <v>330</v>
-      </c>
-      <c r="M57" t="s" s="2">
-        <v>331</v>
-      </c>
-      <c r="N57" s="2"/>
-      <c r="O57" s="2"/>
-      <c r="P57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q57" s="2"/>
-      <c r="R57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X57" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="Y57" t="s" s="2">
-        <v>332</v>
-      </c>
-      <c r="Z57" t="s" s="2">
-        <v>333</v>
-      </c>
-      <c r="AA57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF57" t="s" s="2">
-        <v>329</v>
-      </c>
-      <c r="AG57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AI57" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ57" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AK57" t="s" s="2">
-        <v>325</v>
-      </c>
-      <c r="AL57" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="58" hidden="true">
-      <c r="A58" t="s" s="2">
-        <v>334</v>
-      </c>
-      <c r="B58" t="s" s="2">
-        <v>334</v>
-      </c>
-      <c r="C58" s="2"/>
-      <c r="D58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E58" s="2"/>
-      <c r="F58" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G58" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K58" t="s" s="2">
-        <v>239</v>
-      </c>
-      <c r="L58" t="s" s="2">
-        <v>335</v>
-      </c>
-      <c r="M58" t="s" s="2">
-        <v>336</v>
-      </c>
-      <c r="N58" s="2"/>
-      <c r="O58" s="2"/>
-      <c r="P58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q58" s="2"/>
-      <c r="R58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF58" t="s" s="2">
-        <v>334</v>
-      </c>
-      <c r="AG58" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH58" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI58" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ58" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AK58" t="s" s="2">
-        <v>325</v>
-      </c>
-      <c r="AL58" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="59" hidden="true">
-      <c r="A59" t="s" s="2">
-        <v>337</v>
-      </c>
-      <c r="B59" t="s" s="2">
-        <v>337</v>
-      </c>
-      <c r="C59" s="2"/>
-      <c r="D59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E59" s="2"/>
-      <c r="F59" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G59" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K59" t="s" s="2">
-        <v>338</v>
-      </c>
-      <c r="L59" t="s" s="2">
-        <v>339</v>
-      </c>
-      <c r="M59" t="s" s="2">
-        <v>340</v>
-      </c>
-      <c r="N59" s="2"/>
-      <c r="O59" s="2"/>
-      <c r="P59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q59" s="2"/>
-      <c r="R59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF59" t="s" s="2">
-        <v>337</v>
-      </c>
-      <c r="AG59" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH59" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI59" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ59" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AK59" t="s" s="2">
-        <v>325</v>
-      </c>
-      <c r="AL59" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="60" hidden="true">
-      <c r="A60" t="s" s="2">
-        <v>341</v>
-      </c>
-      <c r="B60" t="s" s="2">
-        <v>341</v>
-      </c>
-      <c r="C60" s="2"/>
-      <c r="D60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E60" s="2"/>
-      <c r="F60" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G60" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K60" t="s" s="2">
-        <v>338</v>
-      </c>
-      <c r="L60" t="s" s="2">
-        <v>342</v>
-      </c>
-      <c r="M60" t="s" s="2">
-        <v>343</v>
-      </c>
-      <c r="N60" s="2"/>
-      <c r="O60" s="2"/>
-      <c r="P60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q60" s="2"/>
-      <c r="R60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF60" t="s" s="2">
-        <v>341</v>
-      </c>
-      <c r="AG60" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH60" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI60" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ60" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AK60" t="s" s="2">
-        <v>325</v>
-      </c>
-      <c r="AL60" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="61" hidden="true">
-      <c r="A61" t="s" s="2">
-        <v>344</v>
-      </c>
-      <c r="B61" t="s" s="2">
-        <v>344</v>
-      </c>
-      <c r="C61" s="2"/>
-      <c r="D61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E61" s="2"/>
-      <c r="F61" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G61" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K61" t="s" s="2">
-        <v>164</v>
-      </c>
-      <c r="L61" t="s" s="2">
-        <v>345</v>
-      </c>
-      <c r="M61" t="s" s="2">
-        <v>346</v>
-      </c>
-      <c r="N61" s="2"/>
-      <c r="O61" s="2"/>
-      <c r="P61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q61" s="2"/>
-      <c r="R61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF61" t="s" s="2">
-        <v>344</v>
-      </c>
-      <c r="AG61" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH61" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI61" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ61" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AK61" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AL61" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="62" hidden="true">
-      <c r="A62" t="s" s="2">
-        <v>347</v>
-      </c>
-      <c r="B62" t="s" s="2">
-        <v>347</v>
-      </c>
-      <c r="C62" s="2"/>
-      <c r="D62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E62" s="2"/>
-      <c r="F62" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G62" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="H62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K62" t="s" s="2">
-        <v>348</v>
-      </c>
-      <c r="L62" t="s" s="2">
-        <v>349</v>
-      </c>
-      <c r="M62" t="s" s="2">
-        <v>350</v>
-      </c>
-      <c r="N62" s="2"/>
-      <c r="O62" t="s" s="2">
-        <v>351</v>
-      </c>
-      <c r="P62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q62" s="2"/>
-      <c r="R62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF62" t="s" s="2">
-        <v>347</v>
-      </c>
-      <c r="AG62" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH62" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AI62" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ62" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AK62" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AL62" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AL62">
+  <autoFilter ref="A1:AL48">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -8168,7 +6529,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI61">
+  <conditionalFormatting sqref="A2:AI47">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>